<commit_message>
feat(budget-planning): add EA blacklist for free planning candidates
</commit_message>
<xml_diff>
--- a/userdata/budget/planning/beauftragungsplanung_config.xlsx
+++ b/userdata/budget/planning/beauftragungsplanung_config.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Daten\Python\vobes_agent_vscode\userdata\budget\planning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE5CBE9A-B66E-47DC-A356-536D1EB99FBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CBD5DE8-DE25-455D-8C42-9BE2C2E705D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="27602" windowHeight="14927" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20060" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Übersicht" sheetId="1" r:id="rId1"/>
     <sheet name="Solver-Parameter" sheetId="2" r:id="rId2"/>
     <sheet name="Firmenziele" sheetId="3" r:id="rId3"/>
     <sheet name="Sondervorgaben" sheetId="4" r:id="rId4"/>
+    <sheet name="EA-Blacklist" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,472 +37,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="143">
-  <si>
-    <t>Parameter</t>
-  </si>
-  <si>
-    <t>Wert</t>
-  </si>
-  <si>
-    <t>Standard</t>
-  </si>
-  <si>
-    <t>Beschreibung</t>
-  </si>
-  <si>
-    <t>stage2_source</t>
-  </si>
-  <si>
-    <t>plan_stage2_results</t>
-  </si>
-  <si>
-    <t>Quelltabelle fuer Stage-2-Ergebnisse in der SQLite-DB. Nicht aendern, es sei denn eine alternative Ergebnis-Tabelle verwendet werden soll.</t>
-  </si>
-  <si>
-    <t>stage2_solver</t>
-  </si>
-  <si>
-    <t>highs</t>
-  </si>
-  <si>
-    <t>Solver-Engine fuer das MIP-Optimierungsproblem. Aktuell wird ausschliesslich 'highs' (HiGHS) unterstuetzt.</t>
-  </si>
-  <si>
-    <t>stage2_activation_penalty</t>
-  </si>
-  <si>
-    <t>600</t>
-  </si>
-  <si>
-    <t>100</t>
-  </si>
-  <si>
-    <t>Jaehrliche Strafkosten (EUR) pro genutztem Entwicklungsauftrag (EA). Hoehere Werte fuehren dazu, dass der Solver weniger verschiedene EAs aktiviert und das Budget auf weniger EAs konzentriert.</t>
-  </si>
-  <si>
-    <t>stage2_quarter_activation_penalty</t>
-  </si>
-  <si>
-    <t>300</t>
-  </si>
-  <si>
-    <t>50</t>
-  </si>
-  <si>
-    <t>Zusaetzliche Strafkosten (EUR) fuer jedes Quartal, in dem ein EA aktiv ist. Hoehere Werte reduzieren die Anzahl der Quartale pro EA und fuehren zu gebuendelteren Beauftragungen.</t>
-  </si>
-  <si>
-    <t>stage2_min_new_order_amount</t>
-  </si>
-  <si>
-    <t>10000</t>
-  </si>
-  <si>
-    <t>Mindestbetrag in EUR fuer neue Beauftragungen. Liegt eine geplante Beauftragung unter diesem Wert, wird sie vom Solver nicht angelegt. Verhindert Kleinstbeauftragungen.</t>
-  </si>
-  <si>
-    <t>stage2_repeat_quarter_penalty</t>
-  </si>
-  <si>
-    <t>200</t>
-  </si>
-  <si>
-    <t>Strafkosten (EUR) wenn dieselbe EA in mehreren aufeinanderfolgenden Quartalen beauftragt wird. Hoehere Werte foerdern eine Rotation der EAs ueber die Quartale.</t>
-  </si>
-  <si>
-    <t>stage2_stop_penalty</t>
-  </si>
-  <si>
-    <t>500</t>
-  </si>
-  <si>
-    <t>Strafkosten (EUR) fuer das Stoppen/Nicht-Fortfuehren eines bestehenden Konzepts (laufende Beauftragung). Schuetzt laufende Beauftragungen vor unnoetiger Unterbrechung.</t>
-  </si>
-  <si>
-    <t>stage2_large_order_penalty</t>
-  </si>
-  <si>
-    <t>700</t>
-  </si>
-  <si>
-    <t>Strafkosten (EUR) fuer Einzelbeauftragungen die den large_order_threshold ueberschreiten. Wirkt gegen zu grosse Einzelpositionen und foerdert eine gleichmaessigere Verteilung.</t>
-  </si>
-  <si>
-    <t>stage2_large_order_threshold</t>
-  </si>
-  <si>
-    <t>40000</t>
-  </si>
-  <si>
-    <t>Schwellenwert in EUR ab dem die large_order_penalty greift. Beauftragungen ueber diesem Betrag erhalten den Strafaufschlag.</t>
-  </si>
-  <si>
-    <t>stage2_existing_small_amount_penalty</t>
-  </si>
-  <si>
-    <t>Reserviert fuer kuenftige Nutzung, derzeit nicht aktiv im Solver. Vorgesehen fuer Strafkosten bei zu kleinen Betraegen auf bestehenden Konzepten.</t>
-  </si>
-  <si>
-    <t>stage2_soft_target_penalty</t>
-  </si>
-  <si>
-    <t>Strafkosten pro EUR Abweichung wenn eine Firma unter ihrem Jahresziel (Firmenziel) bleibt. Hoehere Werte erzwingen eine genauere Einhaltung der Firmenziele.</t>
-  </si>
-  <si>
-    <t>stage2_active_ea_cap_per_quarter</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>Maximale Anzahl aktiver EAs pro Firma und Quartal. 0 = unbegrenzt. Bei Werten &gt; 0 darf eine Firma in einem Quartal hoechstens diese Anzahl verschiedener EAs bedienen.</t>
-  </si>
-  <si>
-    <t>stage2_hard_need_bonus</t>
-  </si>
-  <si>
-    <t>Bonus (negative Strafkosten, EUR) fuer EAs die als 'hart benoetigt' markiert sind (is_hard=1 in Stage-1). Bevorzugt die Zuweisung auf dringend benoetigte EAs.</t>
-  </si>
-  <si>
-    <t>stage2_throughlauf_change_penalty</t>
-  </si>
-  <si>
-    <t>2500</t>
-  </si>
-  <si>
-    <t>Strafkosten pro EUR Reduktion bei laufenden Positionen (Durchlaeufer). Sehr hoher Wert schuetzt bestehende Beauftragungen stark vor Kuerzungen.</t>
-  </si>
-  <si>
-    <t>stage2_special_rule_priority_penalty_step</t>
-  </si>
-  <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>Strafkosten-Stufe (EUR) fuer Firmenprioritaet bei Sondervorgaben. Firma auf Prio 1 bekommt 0 Aufschlag, Prio 2 bekommt 1x diesen Wert, Prio 3 bekommt 2x usw.</t>
-  </si>
-  <si>
-    <t>stage2_special_rule_annual_penalty</t>
-  </si>
-  <si>
-    <t>Strafkosten pro EUR Abweichung vom Sondervorgaben-Zielbetrag. Steuert wie streng der Solver die in den Sondervorgaben definierten FL-Betraege einhält.</t>
-  </si>
-  <si>
-    <t>stage2_global_quarter_undershoot_penalty</t>
-  </si>
-  <si>
-    <t>Strafkosten pro EUR wenn ein Quartal insgesamt unter dem anteiligen Gesamtplan liegt. Verhindert, dass einzelne Quartale zu wenig Budget erhalten.</t>
-  </si>
-  <si>
-    <t>stage2_global_quarter_overshoot_penalty</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>Strafkosten pro EUR wenn ein Quartal insgesamt ueber dem anteiligen Gesamtplan liegt. Bewusst niedrig, da leichte Ueberplanung weniger kritisch ist.</t>
-  </si>
-  <si>
-    <t>stage2_soft_target_overshoot_penalty</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>Strafkosten pro EUR wenn eine Firma ueber ihrem Jahresziel liegt. Niedriger als soft_target_penalty, da Ueberplanung weniger kritisch ist als Unterplanung.</t>
-  </si>
-  <si>
-    <t>stage2_time_limit_seconds</t>
-  </si>
-  <si>
-    <t>120</t>
-  </si>
-  <si>
-    <t>Maximale Rechenzeit des Solvers in Sekunden. Nach Ablauf wird die beste bisher gefundene Loesung verwendet (auch wenn nicht bewiesen optimal).</t>
-  </si>
-  <si>
-    <t>enforce_company_annual_target_consistency</t>
-  </si>
-  <si>
-    <t>true</t>
-  </si>
-  <si>
-    <t>Konsistenzpruefung: Abbruch wenn die Summe der Quartalsziele einer Firma nicht dem Jahresziel entspricht. Sollte normalerweise auf 'true' stehen.</t>
-  </si>
-  <si>
-    <t>btl_opt_refresh</t>
-  </si>
-  <si>
-    <t>replace</t>
-  </si>
-  <si>
-    <t>Aktualisierungsmodus fuer die btl_opt-Tabelle. 'replace' = alle vorhandenen Zeilen loeschen und komplett neu schreiben. Einziger unterstuetzter Modus.</t>
-  </si>
-  <si>
-    <t>Firma</t>
-  </si>
-  <si>
-    <t>Jahresziel_TE</t>
-  </si>
-  <si>
-    <t>Q1</t>
-  </si>
-  <si>
-    <t>Q2</t>
-  </si>
-  <si>
-    <t>Q3</t>
-  </si>
-  <si>
-    <t>Q4</t>
-  </si>
-  <si>
-    <t>Schrittweite</t>
-  </si>
-  <si>
-    <t>Kontrollsumme Quartale</t>
-  </si>
-  <si>
-    <t>4SOFT GMBH MUENCHEN</t>
-  </si>
-  <si>
-    <t>BERTRANDT INGENIEURBUERO GMBH TAPPENBECK</t>
-  </si>
-  <si>
-    <t>EDAG ENGINEERING GMBH WOLFSBURG</t>
-  </si>
-  <si>
-    <t>FES GMBH ZWICKAU/00</t>
-  </si>
-  <si>
-    <t>SUMITOMO ELECTRIC BORDNETZE SE WOLFSBURG</t>
-  </si>
-  <si>
-    <t>THIESEN HARDWARE SOFTW. GMBH WARTENBERG</t>
-  </si>
-  <si>
-    <t>VOITAS ENGINEERING GMBH GEISENFELD</t>
-  </si>
-  <si>
-    <t>VOLKSWAGEN GROUP SERVICES GMBH WOLFSBURG</t>
-  </si>
-  <si>
-    <t>Thema</t>
-  </si>
-  <si>
-    <t>EA</t>
-  </si>
-  <si>
-    <t>EL</t>
-  </si>
-  <si>
-    <t>FL</t>
-  </si>
-  <si>
-    <t>Kadenz</t>
-  </si>
-  <si>
-    <t>Erlaubte_Firmen</t>
-  </si>
-  <si>
-    <t>Prioritaet_Firmen</t>
-  </si>
-  <si>
-    <t>Bemerkung</t>
-  </si>
-  <si>
-    <t>Hinweise</t>
-  </si>
-  <si>
-    <t>PMT</t>
-  </si>
-  <si>
-    <t>43932</t>
-  </si>
-  <si>
-    <t>{'mode': 'hours', 'value': 8449.0, 'display': '8.449h'}</t>
-  </si>
-  <si>
-    <t>quartalsweise</t>
-  </si>
-  <si>
-    <t>4SOFT, THIESEN, VOLKSWAGEN, FES, SUMITOMO</t>
-  </si>
-  <si>
-    <t>FL genehmigt. PMT-ID: 26-011. EL in Stunden!
-100% EL für Ralf, Frank, Michal, Chris
-62% Andreas</t>
-  </si>
-  <si>
-    <t>EL und FL müssen exakt passen!
-EL und FL dürfen nur Quartalsweise beauftragen und werden sehr genau beobachtet.
-Folgende Firmen können auf PMT buchen: 4soft, Thiesen, Volkswagen Group Services, FES, Sumitomo in genau dieser Priorität.
-Achtung: 4soft kann nur auf PMT und Digi-budget gebucht werden!</t>
-  </si>
-  <si>
-    <t>Digi-budget</t>
-  </si>
-  <si>
-    <t>48040</t>
-  </si>
-  <si>
-    <t>{'mode': 'none', 'value': None, 'display': '-'}</t>
-  </si>
-  <si>
-    <t>1. Halbjahr</t>
-  </si>
-  <si>
-    <t>4SOFT, VOLKSWAGEN, FES</t>
-  </si>
-  <si>
-    <t>1. HJ DMU (170T€) + RuleChecker (120T€), aber mind. je 10T€ EL, 2. HJ noch kein Budget</t>
-  </si>
-  <si>
-    <t>FL muss exakt passen! 
-EL kann niedriger sein, darf aber auf keinen Fall höher sein. 
-Werte für 1. HJ müssen auch wirklich im 1.HJ beauftragt werden.
-Folgende Firmen können auf Digi-budget buchen: 4soft, Volkswagen Group Services, FES in genau dieser Priorität.</t>
-  </si>
-  <si>
-    <t>VCTC (KÜE)</t>
-  </si>
-  <si>
-    <t>93037</t>
-  </si>
-  <si>
-    <t>jaehrlich</t>
-  </si>
-  <si>
-    <t>BERTRANDT, EDAG, FES, THIESEN</t>
-  </si>
-  <si>
-    <t>KÜE CMP21D (49T€ &gt; 45T€)</t>
-  </si>
-  <si>
-    <t>Hier nur FL buchen. 
-FL muss exakt passen. 
-FL kann am Stück beauftragt werden (hier keine Quartalsaufteilung notwendig).
-Nur für Bertrandt, EDAG, FES, Thiesen.</t>
-  </si>
-  <si>
-    <t>VCTC (AWS)</t>
-  </si>
-  <si>
-    <t>0055543, 0055544, 0000097</t>
-  </si>
-  <si>
-    <t>AWS  x4 in Summe 45 + 63 + 75 + 63 = 246 (TODO)</t>
-  </si>
-  <si>
-    <t>NE Space Crafter</t>
-  </si>
-  <si>
-    <t>22020</t>
-  </si>
-  <si>
-    <t>{'mode': 'te', 'value': 15.0, 'display': '15'}</t>
-  </si>
-  <si>
-    <t>pro Halbjahr</t>
-  </si>
-  <si>
-    <t>BERTRANDT, EDAG</t>
-  </si>
-  <si>
-    <t>Pro Halbjahr, EL: Armin, Donato, Afshin, TCM</t>
-  </si>
-  <si>
-    <t>EL und FL müssen exakt passen!
-EL und FL müssen hier pro Halbjahr beauftragt werden!
-Nur für Bertrandt und EDAG!</t>
-  </si>
-  <si>
-    <t>NE ID Buzz AD</t>
-  </si>
-  <si>
-    <t>35566</t>
-  </si>
-  <si>
-    <t>pro Quartal</t>
-  </si>
-  <si>
-    <t>Pro Quartal,  EL: Armin, Donato, Afshin, TCM</t>
-  </si>
-  <si>
-    <t>EL und FL müssen exakt passen!
-EL und FL müssen hier pro por Quartal beauftragt werden!
-Nur für Bertrandt und EDAG!</t>
-  </si>
-  <si>
-    <t>MQB@CAE</t>
-  </si>
-  <si>
-    <t>412</t>
-  </si>
-  <si>
-    <t>Ein EA, Budgetadjustierung zugesagt. 323 T€ (2026) + 389 T€ (2027)...</t>
-  </si>
-  <si>
-    <t>Hier nur FL buchen. FL muss exakt passen. FL kann am Stück beauftragt werden (hier keine Quartalsaufteilung notwendig).
-Nur für Bertrandt, EDAG, FES, Thiesen.</t>
-  </si>
-  <si>
-    <t>BIB+China Audi</t>
-  </si>
-  <si>
-    <t>33517</t>
-  </si>
-  <si>
-    <t>EDAG</t>
-  </si>
-  <si>
-    <t>Bib Audi lt. Abmachung 81T€ EL + 238 T€ FL aber intern alles für FL!
-China Audi: 61T€</t>
-  </si>
-  <si>
-    <t>folgende firmen buchen: EDAG
-Zur Not auch andere Firmen/Dienstleister, die woanders abgelehnt werden (prio 2). EA-Target bleibt unverändert.</t>
-  </si>
-  <si>
-    <t>Scania</t>
-  </si>
-  <si>
-    <t>536</t>
-  </si>
-  <si>
-    <t>{'mode': 'manual', 'value': None, 'display': '15000'}</t>
-  </si>
-  <si>
-    <t>keine FL</t>
-  </si>
-  <si>
-    <t>Nur EL. EA Nummer EA536 angelegt und zentrale KÜE 200k€ bestäzigt (TODO)</t>
-  </si>
-  <si>
-    <t>Nur EL. Keine FL.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">ANLEITUNG: Beauftragungsplanung Config Excel
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="211">
+  <si>
+    <t xml:space="preserve">ANLEITUNG: Beauftragungsplanung Config Excel
 =============================================
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
 Diese Excel steuert die automatische Beauftragungsplanung (MIP-Solver).
 Sie besteht aus 4 Tabs — 3 davon sind solver-relevant, dieser Tab ist reine Doku.
 TAB 1: Solver-Parameter
@@ -563,14 +102,661 @@
 Wird NICHT vom Solver ausgewertet — rein dokumentarisch.
 Hier können z.B. Planungsstand, Annahmen und Kontextinfos notiert werden.
 </t>
-    </r>
+  </si>
+  <si>
+    <t>Parameter</t>
+  </si>
+  <si>
+    <t>Wert</t>
+  </si>
+  <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>Beschreibung</t>
+  </si>
+  <si>
+    <t>stage2_source</t>
+  </si>
+  <si>
+    <t>plan_stage2_results</t>
+  </si>
+  <si>
+    <t>Quelltabelle fuer Stage-2-Ergebnisse in der SQLite-DB. Nicht aendern, es sei denn eine alternative Ergebnis-Tabelle verwendet werden soll.</t>
+  </si>
+  <si>
+    <t>stage2_solver</t>
+  </si>
+  <si>
+    <t>highs</t>
+  </si>
+  <si>
+    <t>Solver-Engine fuer das MIP-Optimierungsproblem. Aktuell wird ausschliesslich 'highs' (HiGHS) unterstuetzt.</t>
+  </si>
+  <si>
+    <t>stage2_activation_penalty</t>
+  </si>
+  <si>
+    <t>600</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>Jaehrliche Strafkosten (EUR) pro genutztem Entwicklungsauftrag (EA). Hoehere Werte fuehren dazu, dass der Solver weniger verschiedene EAs aktiviert und das Budget auf weniger EAs konzentriert.</t>
+  </si>
+  <si>
+    <t>stage2_quarter_activation_penalty</t>
+  </si>
+  <si>
+    <t>300</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>Zusaetzliche Strafkosten (EUR) fuer jedes Quartal, in dem ein EA aktiv ist. Hoehere Werte reduzieren die Anzahl der Quartale pro EA und fuehren zu gebuendelteren Beauftragungen.</t>
+  </si>
+  <si>
+    <t>stage2_min_new_order_amount</t>
+  </si>
+  <si>
+    <t>10000</t>
+  </si>
+  <si>
+    <t>Mindestbetrag in EUR fuer neue Beauftragungen. Liegt eine geplante Beauftragung unter diesem Wert, wird sie vom Solver nicht angelegt. Verhindert Kleinstbeauftragungen.</t>
+  </si>
+  <si>
+    <t>stage2_repeat_quarter_penalty</t>
+  </si>
+  <si>
+    <t>200</t>
+  </si>
+  <si>
+    <t>Strafkosten (EUR) wenn dieselbe EA in mehreren aufeinanderfolgenden Quartalen beauftragt wird. Hoehere Werte foerdern eine Rotation der EAs ueber die Quartale.</t>
+  </si>
+  <si>
+    <t>stage2_stop_penalty</t>
+  </si>
+  <si>
+    <t>500</t>
+  </si>
+  <si>
+    <t>Strafkosten (EUR) fuer das Stoppen/Nicht-Fortfuehren eines bestehenden Konzepts (laufende Beauftragung). Schuetzt laufende Beauftragungen vor unnoetiger Unterbrechung.</t>
+  </si>
+  <si>
+    <t>stage2_large_order_penalty</t>
+  </si>
+  <si>
+    <t>700</t>
+  </si>
+  <si>
+    <t>Strafkosten (EUR) fuer Einzelbeauftragungen die den large_order_threshold ueberschreiten. Wirkt gegen zu grosse Einzelpositionen und foerdert eine gleichmaessigere Verteilung.</t>
+  </si>
+  <si>
+    <t>stage2_large_order_threshold</t>
+  </si>
+  <si>
+    <t>40000</t>
+  </si>
+  <si>
+    <t>Schwellenwert in EUR ab dem die large_order_penalty greift. Beauftragungen ueber diesem Betrag erhalten den Strafaufschlag.</t>
+  </si>
+  <si>
+    <t>stage2_existing_small_amount_penalty</t>
+  </si>
+  <si>
+    <t>Reserviert fuer kuenftige Nutzung, derzeit nicht aktiv im Solver. Vorgesehen fuer Strafkosten bei zu kleinen Betraegen auf bestehenden Konzepten.</t>
+  </si>
+  <si>
+    <t>stage2_soft_target_penalty</t>
+  </si>
+  <si>
+    <t>Strafkosten pro EUR Abweichung wenn eine Firma unter ihrem Jahresziel (Firmenziel) bleibt. Hoehere Werte erzwingen eine genauere Einhaltung der Firmenziele.</t>
+  </si>
+  <si>
+    <t>stage2_active_ea_cap_per_quarter</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>Maximale Anzahl aktiver EAs pro Firma und Quartal. 0 = unbegrenzt. Bei Werten &gt; 0 darf eine Firma in einem Quartal hoechstens diese Anzahl verschiedener EAs bedienen.</t>
+  </si>
+  <si>
+    <t>stage2_hard_need_bonus</t>
+  </si>
+  <si>
+    <t>Bonus (negative Strafkosten, EUR) fuer EAs die als 'hart benoetigt' markiert sind (is_hard=1 in Stage-1). Bevorzugt die Zuweisung auf dringend benoetigte EAs.</t>
+  </si>
+  <si>
+    <t>stage2_throughlauf_change_penalty</t>
+  </si>
+  <si>
+    <t>2500</t>
+  </si>
+  <si>
+    <t>Strafkosten pro EUR Reduktion bei laufenden Positionen (Durchlaeufer). Sehr hoher Wert schuetzt bestehende Beauftragungen stark vor Kuerzungen.</t>
+  </si>
+  <si>
+    <t>stage2_special_rule_priority_penalty_step</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>Strafkosten-Stufe (EUR) fuer Firmenprioritaet bei Sondervorgaben. Firma auf Prio 1 bekommt 0 Aufschlag, Prio 2 bekommt 1x diesen Wert, Prio 3 bekommt 2x usw.</t>
+  </si>
+  <si>
+    <t>stage2_special_rule_annual_penalty</t>
+  </si>
+  <si>
+    <t>Strafkosten pro EUR Abweichung vom Sondervorgaben-Zielbetrag. Steuert wie streng der Solver die in den Sondervorgaben definierten FL-Betraege einhält.</t>
+  </si>
+  <si>
+    <t>stage2_global_quarter_undershoot_penalty</t>
+  </si>
+  <si>
+    <t>Strafkosten pro EUR wenn ein Quartal insgesamt unter dem anteiligen Gesamtplan liegt. Verhindert, dass einzelne Quartale zu wenig Budget erhalten.</t>
+  </si>
+  <si>
+    <t>stage2_global_quarter_overshoot_penalty</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>Strafkosten pro EUR wenn ein Quartal insgesamt ueber dem anteiligen Gesamtplan liegt. Bewusst niedrig, da leichte Ueberplanung weniger kritisch ist.</t>
+  </si>
+  <si>
+    <t>stage2_soft_target_overshoot_penalty</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Strafkosten pro EUR wenn eine Firma ueber ihrem Jahresziel liegt. Niedriger als soft_target_penalty, da Ueberplanung weniger kritisch ist als Unterplanung.</t>
+  </si>
+  <si>
+    <t>stage2_time_limit_seconds</t>
+  </si>
+  <si>
+    <t>120</t>
+  </si>
+  <si>
+    <t>Maximale Rechenzeit des Solvers in Sekunden. Nach Ablauf wird die beste bisher gefundene Loesung verwendet (auch wenn nicht bewiesen optimal).</t>
+  </si>
+  <si>
+    <t>enforce_company_annual_target_consistency</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>Konsistenzpruefung: Abbruch wenn die Summe der Quartalsziele einer Firma nicht dem Jahresziel entspricht. Sollte normalerweise auf 'true' stehen.</t>
+  </si>
+  <si>
+    <t>btl_opt_refresh</t>
+  </si>
+  <si>
+    <t>replace</t>
+  </si>
+  <si>
+    <t>Aktualisierungsmodus fuer die btl_opt-Tabelle. 'replace' = alle vorhandenen Zeilen loeschen und komplett neu schreiben. Einziger unterstuetzter Modus.</t>
+  </si>
+  <si>
+    <t>Firma</t>
+  </si>
+  <si>
+    <t>Jahresziel_TE</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>Q3</t>
+  </si>
+  <si>
+    <t>Q4</t>
+  </si>
+  <si>
+    <t>Schrittweite</t>
+  </si>
+  <si>
+    <t>Kontrollsumme Quartale</t>
+  </si>
+  <si>
+    <t>4SOFT GMBH MUENCHEN</t>
+  </si>
+  <si>
+    <t>BERTRANDT INGENIEURBUERO GMBH TAPPENBECK</t>
+  </si>
+  <si>
+    <t>EDAG ENGINEERING GMBH WOLFSBURG</t>
+  </si>
+  <si>
+    <t>FES GMBH ZWICKAU/00</t>
+  </si>
+  <si>
+    <t>SUMITOMO ELECTRIC BORDNETZE SE WOLFSBURG</t>
+  </si>
+  <si>
+    <t>THIESEN HARDWARE SOFTW. GMBH WARTENBERG</t>
+  </si>
+  <si>
+    <t>VOITAS ENGINEERING GMBH GEISENFELD</t>
+  </si>
+  <si>
+    <t>VOLKSWAGEN GROUP SERVICES GMBH WOLFSBURG</t>
+  </si>
+  <si>
+    <t>Thema</t>
+  </si>
+  <si>
+    <t>EA</t>
+  </si>
+  <si>
+    <t>EL</t>
+  </si>
+  <si>
+    <t>FL</t>
+  </si>
+  <si>
+    <t>Kadenz</t>
+  </si>
+  <si>
+    <t>Erlaubte_Firmen</t>
+  </si>
+  <si>
+    <t>Prioritaet_Firmen</t>
+  </si>
+  <si>
+    <t>Bemerkung</t>
+  </si>
+  <si>
+    <t>Hinweise</t>
+  </si>
+  <si>
+    <t>PMT</t>
+  </si>
+  <si>
+    <t>43932</t>
+  </si>
+  <si>
+    <t>{'mode': 'hours', 'value': 8449.0, 'display': '8.449h'}</t>
+  </si>
+  <si>
+    <t>quartalsweise</t>
+  </si>
+  <si>
+    <t>4SOFT, THIESEN, VOLKSWAGEN, FES, SUMITOMO</t>
+  </si>
+  <si>
+    <t>FL genehmigt. PMT-ID: 26-011. EL in Stunden!
+100% EL für Ralf, Frank, Michal, Chris
+62% Andreas</t>
+  </si>
+  <si>
+    <t>EL und FL müssen exakt passen!
+EL und FL dürfen nur Quartalsweise beauftragen und werden sehr genau beobachtet.
+Folgende Firmen können auf PMT buchen: 4soft, Thiesen, Volkswagen Group Services, FES, Sumitomo in genau dieser Priorität.
+Achtung: 4soft kann nur auf PMT und Digi-budget gebucht werden!</t>
+  </si>
+  <si>
+    <t>Digi-budget</t>
+  </si>
+  <si>
+    <t>48040</t>
+  </si>
+  <si>
+    <t>{'mode': 'none', 'value': None, 'display': '-'}</t>
+  </si>
+  <si>
+    <t>1. Halbjahr</t>
+  </si>
+  <si>
+    <t>4SOFT, VOLKSWAGEN, FES</t>
+  </si>
+  <si>
+    <t>1. HJ DMU (170T€) + RuleChecker (120T€), aber mind. je 10T€ EL, 2. HJ noch kein Budget</t>
+  </si>
+  <si>
+    <t>FL muss exakt passen! 
+EL kann niedriger sein, darf aber auf keinen Fall höher sein. 
+Werte für 1. HJ müssen auch wirklich im 1.HJ beauftragt werden.
+Folgende Firmen können auf Digi-budget buchen: 4soft, Volkswagen Group Services, FES in genau dieser Priorität.</t>
+  </si>
+  <si>
+    <t>VCTC (KÜE)</t>
+  </si>
+  <si>
+    <t>93037</t>
+  </si>
+  <si>
+    <t>jaehrlich</t>
+  </si>
+  <si>
+    <t>BERTRANDT, EDAG, FES, THIESEN</t>
+  </si>
+  <si>
+    <t>KÜE CMP21D (49T€ &gt; 45T€)</t>
+  </si>
+  <si>
+    <t>Hier nur FL buchen. 
+FL muss exakt passen. 
+FL kann am Stück beauftragt werden (hier keine Quartalsaufteilung notwendig).
+Nur für Bertrandt, EDAG, FES, Thiesen.</t>
+  </si>
+  <si>
+    <t>VCTC (AWS)</t>
+  </si>
+  <si>
+    <t>0055543, 0055544, 0000097</t>
+  </si>
+  <si>
+    <t>AWS  x4 in Summe 45 + 63 + 75 + 63 = 246 (TODO)</t>
+  </si>
+  <si>
+    <t>NE Space Crafter</t>
+  </si>
+  <si>
+    <t>22020</t>
+  </si>
+  <si>
+    <t>{'mode': 'te', 'value': 15.0, 'display': '15'}</t>
+  </si>
+  <si>
+    <t>pro Halbjahr</t>
+  </si>
+  <si>
+    <t>BERTRANDT, EDAG</t>
+  </si>
+  <si>
+    <t>Pro Halbjahr, EL: Armin, Donato, Afshin, TCM</t>
+  </si>
+  <si>
+    <t>EL und FL müssen exakt passen!
+EL und FL müssen hier pro Halbjahr beauftragt werden!
+Nur für Bertrandt und EDAG!</t>
+  </si>
+  <si>
+    <t>NE ID Buzz AD</t>
+  </si>
+  <si>
+    <t>35566</t>
+  </si>
+  <si>
+    <t>pro Quartal</t>
+  </si>
+  <si>
+    <t>Pro Quartal,  EL: Armin, Donato, Afshin, TCM</t>
+  </si>
+  <si>
+    <t>EL und FL müssen exakt passen!
+EL und FL müssen hier pro por Quartal beauftragt werden!
+Nur für Bertrandt und EDAG!</t>
+  </si>
+  <si>
+    <t>MQB@CAE</t>
+  </si>
+  <si>
+    <t>412</t>
+  </si>
+  <si>
+    <t>Ein EA, Budgetadjustierung zugesagt. 323 T€ (2026) + 389 T€ (2027)...</t>
+  </si>
+  <si>
+    <t>Hier nur FL buchen. FL muss exakt passen. FL kann am Stück beauftragt werden (hier keine Quartalsaufteilung notwendig).
+Nur für Bertrandt, EDAG, FES, Thiesen.</t>
+  </si>
+  <si>
+    <t>BIB+China Audi</t>
+  </si>
+  <si>
+    <t>33517</t>
+  </si>
+  <si>
+    <t>EDAG</t>
+  </si>
+  <si>
+    <t>Bib Audi lt. Abmachung 81T€ EL + 238 T€ FL aber intern alles für FL!
+China Audi: 61T€</t>
+  </si>
+  <si>
+    <t>folgende firmen buchen: EDAG
+Zur Not auch andere Firmen/Dienstleister, die woanders abgelehnt werden (prio 2). EA-Target bleibt unverändert.</t>
+  </si>
+  <si>
+    <t>Scania</t>
+  </si>
+  <si>
+    <t>536</t>
+  </si>
+  <si>
+    <t>{'mode': 'manual', 'value': None, 'display': '15000'}</t>
+  </si>
+  <si>
+    <t>keine FL</t>
+  </si>
+  <si>
+    <t>Nur EL. EA Nummer EA536 angelegt und zentrale KÜE 200k€ bestäzigt (TODO)</t>
+  </si>
+  <si>
+    <t>Nur EL. Keine FL.</t>
+  </si>
+  <si>
+    <t>EA-Bezeichnung</t>
+  </si>
+  <si>
+    <t>Grund</t>
+  </si>
+  <si>
+    <t>90741</t>
+  </si>
+  <si>
+    <t>Nachträgliche Projektkostenzuordnung</t>
+  </si>
+  <si>
+    <t>9999999</t>
+  </si>
+  <si>
+    <t>Rest/Sachgemeinkosten</t>
+  </si>
+  <si>
+    <t>10933</t>
+  </si>
+  <si>
+    <t>Baukasten PKO Maßnahmen SOP 2027-2029</t>
+  </si>
+  <si>
+    <t>87813</t>
+  </si>
+  <si>
+    <t>Modul Innenspiegel mit MIK MQB27</t>
+  </si>
+  <si>
+    <t>TEDigitalisierung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nachträgliche Projektkostenzuordnung                        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baukasten PKO Maßnahmen SOP 2027-2029                       </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modul Innenspiegel mit MIK MQB27                            </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TE-PMT Mechanikentwicklung                                  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arbeiten für FE-externe EK                                  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">VESmart Exterieur                                           </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SPACE -e-Crafter (MEB)                                      </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modul Ladedosen AC &amp; Combo/DLD/DC Gen.4                     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PKW Aktionsmodelle VW                                       </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEDigitalisierung                                           </t>
+  </si>
+  <si>
+    <t xml:space="preserve">VE Vision Zero                                              </t>
+  </si>
+  <si>
+    <t xml:space="preserve">VESmart Interieur                                           </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weltmodul Klapplehne                                        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAD/CAT Methoden- und Applikationsentw.                     </t>
+  </si>
+  <si>
+    <t>Grundlast und PV-Wechsel Hut MP MQBevo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VE Pilotiertes Fahren                                       </t>
+  </si>
+  <si>
+    <t>Kreislauffähigkeit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VE Prototypenfreie phys. Absicherung                        </t>
+  </si>
+  <si>
+    <t>MQB@CEA C6b Plattformumfänge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TE-PMT Anforderungsmanagement                               </t>
+  </si>
+  <si>
+    <t xml:space="preserve">VE Virt. Entw. el. Antriebe                                 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">VE Intelligenter Leichtbau                                  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MIK Multifunktionsinnenraumkamera                           </t>
+  </si>
+  <si>
+    <t xml:space="preserve">HV Wasserheizer KKH06                                       </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modul Thermo-System MQB/MEB                                 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Klimafunktionssoftware SSP                                  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">VE Smart Cockpit &amp; Intuitive Usability                      </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Klimaheizgerät SSPals Einzelmodul                           </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSC Entscheidungen                                          </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auftragsentwicklung MEB31 Skoda 7S EU                       </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SB Module EE                                                </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SB Einzelmodule Thermo-System                               </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plattforminteg. C2P Optima Next Level                       </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Produkthaftpflichtfaelle                                    </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TE-Effizienzprogramm -Pitchday Themen                       </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MQBevo BCM Re-Design                                        </t>
+  </si>
+  <si>
+    <t>Konzept MQBevo AmainSUV NAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meßtechnik Sicherheitsversuch Plattformübergreife           </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MQBevo - Funktionserweiterung MJW24/28                      </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ModulTBK Sitzanlagen                                        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MQB Ertüchtigung funktionale Sicherheit                     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">VE Kompetenzentwicklung                                     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lenkrad Gen.X China                                         </t>
+  </si>
+  <si>
+    <t>Nur für VE/Digitaliseirungsprojekte</t>
+  </si>
+  <si>
+    <t>Vorhalt (nur für Fremdleistung! / EK-intern)</t>
+  </si>
+  <si>
+    <t>Nur Vorhalt. Soll wg. VS nicht beplant werden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SB MQB27/37/41/48/SUV inkl. BEV/PHEV                        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SB VW53X Hut                                                </t>
+  </si>
+  <si>
+    <t xml:space="preserve">VW416/6B-SUVe 5S FBU EU                                     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SSP31B NAR                                                  </t>
+  </si>
+  <si>
+    <t>VW423/1CS_B – B Sedan</t>
+  </si>
+  <si>
+    <t>VW423/1CS_E – B Sedan – EREV</t>
+  </si>
+  <si>
+    <t>CSP31D EREV (B NB)</t>
+  </si>
+  <si>
+    <t>VW326/6CS_B – A+ SUV – EREV</t>
+  </si>
+  <si>
+    <t>CSP31B EREV (A+)</t>
+  </si>
+  <si>
+    <t>Projektleiter hat angelehnt</t>
+  </si>
+  <si>
+    <t>Spezial-EA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -600,13 +786,19 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -646,8 +838,19 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -681,11 +884,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -745,9 +963,31 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1057,18 +1297,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="261.10000000000002" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
-        <v>142</v>
+      <c r="A1" s="23" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="261.10000000000002" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="21"/>
+      <c r="A2" s="24"/>
     </row>
     <row r="3" spans="1:1" ht="261.10000000000002" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="21"/>
+      <c r="A3" s="24"/>
     </row>
     <row r="4" spans="1:1" ht="261.10000000000002" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="21"/>
+      <c r="A4" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1076,7 +1316,7 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
-    <oddHeader>&amp;L&amp;"Arial"&amp;8&amp;K000000 INTERNAL&amp;1#_x000D_&amp;"Calibri"&amp;11&amp;K000000&amp;"Calibri"&amp;11&amp;K000000&amp;"Arial"&amp;1 &amp;K000000 INTERNAL#_x000D_</oddHeader>
+    <oddHeader>&amp;L&amp;"Arial"&amp;8&amp;K000000 INTERNAL&amp;1#_x000D_&amp;"Calibri"&amp;11&amp;K000000&amp;"Calibri"&amp;11&amp;K000000&amp;"Calibri"&amp;11&amp;K000000&amp;"Arial"&amp;1 &amp;K000000 INTERNAL#_x000D_</oddHeader>
   </headerFooter>
 </worksheet>
 </file>
@@ -1089,330 +1329,330 @@
     <col min="1" max="1" width="43" style="5" customWidth="1"/>
     <col min="2" max="3" width="21" style="5" customWidth="1"/>
     <col min="4" max="4" width="78.140625" style="14" customWidth="1"/>
-    <col min="5" max="6" width="9.140625" style="5" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="5"/>
+    <col min="5" max="7" width="9.140625" style="5" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C1" s="19" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="28.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="28.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="42.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="42.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="42.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="28.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="42.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="42.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="28.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="28.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="42.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="42.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="28.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="28.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="28.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="28.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="28.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="28.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="28.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="28.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B21" s="16">
         <v>200</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="28.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="28.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1423,7 +1663,7 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
-    <oddHeader>&amp;L&amp;"Arial"&amp;8&amp;K000000 INTERNAL&amp;1#_x000D_&amp;"Calibri"&amp;11&amp;K000000&amp;"Calibri"&amp;11&amp;K000000&amp;"Arial"&amp;1 &amp;K000000 INTERNAL#_x000D_</oddHeader>
+    <oddHeader>&amp;L&amp;"Arial"&amp;8&amp;K000000 INTERNAL&amp;1#_x000D_&amp;"Calibri"&amp;11&amp;K000000&amp;"Calibri"&amp;11&amp;K000000&amp;"Calibri"&amp;11&amp;K000000&amp;"Arial"&amp;1 &amp;K000000 INTERNAL#_x000D_</oddHeader>
   </headerFooter>
 </worksheet>
 </file>
@@ -1442,33 +1682,33 @@
   <sheetData>
     <row r="1" spans="1:8" ht="28.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B2" s="10">
         <v>974</v>
@@ -1495,7 +1735,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B3" s="10">
         <v>905</v>
@@ -1522,7 +1762,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B4" s="10">
         <v>1088</v>
@@ -1549,7 +1789,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B5" s="10">
         <v>478</v>
@@ -1576,7 +1816,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B6" s="10">
         <v>156</v>
@@ -1603,7 +1843,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B7" s="10">
         <v>551</v>
@@ -1630,7 +1870,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B8" s="10">
         <v>0</v>
@@ -1657,7 +1897,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B9" s="10">
         <v>281</v>
@@ -1685,7 +1925,7 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
-    <oddHeader>&amp;L&amp;"Arial"&amp;8&amp;K000000 INTERNAL&amp;1#_x000D_&amp;"Calibri"&amp;11&amp;K000000&amp;"Calibri"&amp;11&amp;K000000&amp;"Arial"&amp;1 &amp;K000000 INTERNAL#_x000D_</oddHeader>
+    <oddHeader>&amp;L&amp;"Arial"&amp;8&amp;K000000 INTERNAL&amp;1#_x000D_&amp;"Calibri"&amp;11&amp;K000000&amp;"Calibri"&amp;11&amp;K000000&amp;"Calibri"&amp;11&amp;K000000&amp;"Arial"&amp;1 &amp;K000000 INTERNAL#_x000D_</oddHeader>
   </headerFooter>
 </worksheet>
 </file>
@@ -1701,277 +1941,854 @@
     <col min="7" max="7" width="30.85546875" style="3" customWidth="1"/>
     <col min="8" max="8" width="46" style="3" customWidth="1"/>
     <col min="9" max="9" width="67.42578125" style="3" customWidth="1"/>
-    <col min="10" max="10" width="18" style="3" customWidth="1"/>
-    <col min="11" max="16384" width="18" style="3"/>
+    <col min="10" max="11" width="18" style="3" customWidth="1"/>
+    <col min="12" max="16384" width="18" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C1" s="20" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H1" s="20" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I1" s="20" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="85.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D2" s="18">
         <v>1048</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="71.3" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D3" s="18">
         <v>290</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="71.3" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D4" s="18">
         <v>45</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="71.3" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D5" s="18">
         <v>201</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="42.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D6" s="18">
         <v>150</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="42.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D7" s="18">
         <v>150</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="42.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D8" s="18">
         <v>323</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="42.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="42.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
-    <oddHeader>&amp;L&amp;"Arial"&amp;8&amp;K000000 INTERNAL&amp;1#_x000D_&amp;"Calibri"&amp;11&amp;K000000&amp;"Calibri"&amp;11&amp;K000000&amp;"Arial"&amp;1 &amp;K000000 INTERNAL#_x000D_</oddHeader>
+    <oddHeader>&amp;L&amp;"Arial"&amp;8&amp;K000000 INTERNAL&amp;1#_x000D_&amp;"Calibri"&amp;11&amp;K000000&amp;"Calibri"&amp;11&amp;K000000&amp;"Calibri"&amp;11&amp;K000000&amp;"Arial"&amp;1 &amp;K000000 INTERNAL#_x000D_</oddHeader>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:C59"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14" style="27" customWidth="1"/>
+    <col min="2" max="2" width="45.5703125" customWidth="1"/>
+    <col min="3" max="3" width="67.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="21" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1" s="21" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="26" t="s">
+        <v>101</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="C2" s="22" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="28">
+        <v>5555555</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>198</v>
+      </c>
+      <c r="C3" s="22" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="26" t="s">
+        <v>145</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>146</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="26" t="s">
+        <v>147</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="30">
+        <v>42920</v>
+      </c>
+      <c r="B6" s="31" t="s">
+        <v>200</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="30">
+        <v>34655</v>
+      </c>
+      <c r="B7" s="31" t="s">
+        <v>201</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="30">
+        <v>237</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>202</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="30">
+        <v>170</v>
+      </c>
+      <c r="B9" s="31" t="s">
+        <v>203</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="30">
+        <v>65</v>
+      </c>
+      <c r="B10" s="31" t="s">
+        <v>204</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="30">
+        <v>358</v>
+      </c>
+      <c r="B11" s="31" t="s">
+        <v>205</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="30">
+        <v>357</v>
+      </c>
+      <c r="B12" s="31" t="s">
+        <v>206</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="30">
+        <v>398</v>
+      </c>
+      <c r="B13" s="31" t="s">
+        <v>207</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="30">
+        <v>421</v>
+      </c>
+      <c r="B14" s="31" t="s">
+        <v>208</v>
+      </c>
+      <c r="C14" s="22" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="26" t="s">
+        <v>149</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="C15" s="22"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="26" t="s">
+        <v>151</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="C16" s="22"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="26">
+        <v>90741</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>154</v>
+      </c>
+      <c r="C17" s="22"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="26">
+        <v>10933</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="C18" s="22"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="26">
+        <v>87813</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>156</v>
+      </c>
+      <c r="C19" s="22"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="26">
+        <v>43932</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="C20" s="22"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="26">
+        <v>33517</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="C21" s="22"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="26">
+        <v>62819</v>
+      </c>
+      <c r="B22" s="22" t="s">
+        <v>159</v>
+      </c>
+      <c r="C22" s="22"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="26">
+        <v>22020</v>
+      </c>
+      <c r="B23" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="C23" s="22"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="26">
+        <v>87808</v>
+      </c>
+      <c r="B24" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="C24" s="22"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="26">
+        <v>56900</v>
+      </c>
+      <c r="B25" s="22" t="s">
+        <v>162</v>
+      </c>
+      <c r="C25" s="22"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="26">
+        <v>48040</v>
+      </c>
+      <c r="B26" s="22" t="s">
+        <v>163</v>
+      </c>
+      <c r="C26" s="22"/>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="26">
+        <v>62816</v>
+      </c>
+      <c r="B27" s="22" t="s">
+        <v>164</v>
+      </c>
+      <c r="C27" s="22"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="26">
+        <v>62815</v>
+      </c>
+      <c r="B28" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="C28" s="22"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="26">
+        <v>87800</v>
+      </c>
+      <c r="B29" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="C29" s="22"/>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="26">
+        <v>48018</v>
+      </c>
+      <c r="B30" s="22" t="s">
+        <v>167</v>
+      </c>
+      <c r="C30" s="22"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="26">
+        <v>395</v>
+      </c>
+      <c r="B31" s="22" t="s">
+        <v>168</v>
+      </c>
+      <c r="C31" s="22"/>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="26">
+        <v>62835</v>
+      </c>
+      <c r="B32" s="22" t="s">
+        <v>169</v>
+      </c>
+      <c r="C32" s="22"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="26">
+        <v>273</v>
+      </c>
+      <c r="B33" s="22" t="s">
+        <v>170</v>
+      </c>
+      <c r="C33" s="22"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="26">
+        <v>48204</v>
+      </c>
+      <c r="B34" s="22" t="s">
+        <v>171</v>
+      </c>
+      <c r="C34" s="22"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="26">
+        <v>412</v>
+      </c>
+      <c r="B35" s="22" t="s">
+        <v>172</v>
+      </c>
+      <c r="C35" s="22"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="26">
+        <v>43923</v>
+      </c>
+      <c r="B36" s="22" t="s">
+        <v>173</v>
+      </c>
+      <c r="C36" s="22"/>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="26">
+        <v>62823</v>
+      </c>
+      <c r="B37" s="22" t="s">
+        <v>174</v>
+      </c>
+      <c r="C37" s="22"/>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="26">
+        <v>62802</v>
+      </c>
+      <c r="B38" s="22" t="s">
+        <v>175</v>
+      </c>
+      <c r="C38" s="22"/>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="26">
+        <v>87445</v>
+      </c>
+      <c r="B39" s="22" t="s">
+        <v>176</v>
+      </c>
+      <c r="C39" s="22"/>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="26">
+        <v>87779</v>
+      </c>
+      <c r="B40" s="22" t="s">
+        <v>177</v>
+      </c>
+      <c r="C40" s="22"/>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="26">
+        <v>87814</v>
+      </c>
+      <c r="B41" s="22" t="s">
+        <v>178</v>
+      </c>
+      <c r="C41" s="22"/>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="26">
+        <v>87778</v>
+      </c>
+      <c r="B42" s="22" t="s">
+        <v>179</v>
+      </c>
+      <c r="C42" s="22"/>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="26">
+        <v>62814</v>
+      </c>
+      <c r="B43" s="22" t="s">
+        <v>180</v>
+      </c>
+      <c r="C43" s="22"/>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="26">
+        <v>87804</v>
+      </c>
+      <c r="B44" s="22" t="s">
+        <v>181</v>
+      </c>
+      <c r="C44" s="22"/>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="26">
+        <v>9619</v>
+      </c>
+      <c r="B45" s="22" t="s">
+        <v>182</v>
+      </c>
+      <c r="C45" s="22"/>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" s="26">
+        <v>43743</v>
+      </c>
+      <c r="B46" s="22" t="s">
+        <v>183</v>
+      </c>
+      <c r="C46" s="22"/>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" s="26">
+        <v>87343</v>
+      </c>
+      <c r="B47" s="22" t="s">
+        <v>184</v>
+      </c>
+      <c r="C47" s="22"/>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" s="26">
+        <v>87822</v>
+      </c>
+      <c r="B48" s="22" t="s">
+        <v>185</v>
+      </c>
+      <c r="C48" s="22"/>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="26">
+        <v>43904</v>
+      </c>
+      <c r="B49" s="22" t="s">
+        <v>186</v>
+      </c>
+      <c r="C49" s="22"/>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="26">
+        <v>33501</v>
+      </c>
+      <c r="B50" s="22" t="s">
+        <v>187</v>
+      </c>
+      <c r="C50" s="22"/>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="26">
+        <v>10938</v>
+      </c>
+      <c r="B51" s="22" t="s">
+        <v>188</v>
+      </c>
+      <c r="C51" s="22"/>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="26">
+        <v>43866</v>
+      </c>
+      <c r="B52" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="C52" s="22"/>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="26">
+        <v>245</v>
+      </c>
+      <c r="B53" s="22" t="s">
+        <v>190</v>
+      </c>
+      <c r="C53" s="22"/>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="26">
+        <v>35005</v>
+      </c>
+      <c r="B54" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="C54" s="22"/>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="26">
+        <v>45028</v>
+      </c>
+      <c r="B55" s="22" t="s">
+        <v>192</v>
+      </c>
+      <c r="C55" s="22"/>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="26">
+        <v>87441</v>
+      </c>
+      <c r="B56" s="22" t="s">
+        <v>193</v>
+      </c>
+      <c r="C56" s="22"/>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="26">
+        <v>43798</v>
+      </c>
+      <c r="B57" s="22" t="s">
+        <v>194</v>
+      </c>
+      <c r="C57" s="22"/>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" s="26">
+        <v>62800</v>
+      </c>
+      <c r="B58" s="22" t="s">
+        <v>195</v>
+      </c>
+      <c r="C58" s="22"/>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" s="26">
+        <v>87782</v>
+      </c>
+      <c r="B59" s="22" t="s">
+        <v>196</v>
+      </c>
+      <c r="C59" s="22"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;"Arial"&amp;8&amp;K000000 INTERNAL&amp;1#_x000D_</oddHeader>
   </headerFooter>
 </worksheet>
 </file>

</xml_diff>